<commit_message>
actualizacion al 7 de octubre de las listas
</commit_message>
<xml_diff>
--- a/inasistencias-4b-ElectYsistDeComTP/alumnos-4b-ElectroYSistDeCom.xlsx
+++ b/inasistencias-4b-ElectYsistDeComTP/alumnos-4b-ElectroYSistDeCom.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="104">
   <si>
     <t xml:space="preserve">nro</t>
   </si>
@@ -53,6 +53,18 @@
     <t xml:space="preserve">Val Ped</t>
   </si>
   <si>
+    <t xml:space="preserve">Nota-EC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nota proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Victoria</t>
   </si>
   <si>
@@ -80,6 +92,12 @@
     <t xml:space="preserve">emprolijar la cajita</t>
   </si>
   <si>
+    <t xml:space="preserve">traer cajita, traer ladron de joules, video con todo andando</t>
+  </si>
+  <si>
+    <t xml:space="preserve">probarlo a full</t>
+  </si>
+  <si>
     <t xml:space="preserve">Eugenia</t>
   </si>
   <si>
@@ -140,7 +158,10 @@
     <t xml:space="preserve">soldar los componentes , todo unto en una cajita. llevar el modelo al video, si funciona mantenemos el 10</t>
   </si>
   <si>
-    <t xml:space="preserve">ttradr un video donde se me mida con un tester la generacion de energia, ver de hacer un ladron de joules y un diodo</t>
+    <t xml:space="preserve">traer un video donde se me mida con un tester la generacion de energia, ver de hacer un ladron de joules y un diodo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">armar la otra mitad del ladron y generar la tension prometida  y grabar video</t>
   </si>
   <si>
     <t xml:space="preserve">Julieta</t>
@@ -182,6 +203,9 @@
     <t xml:space="preserve">armar un video con la generacion y la carga de la bateria</t>
   </si>
   <si>
+    <t xml:space="preserve">falta la carga de la bateria, agregar al video</t>
+  </si>
+  <si>
     <t xml:space="preserve">Farid Emir</t>
   </si>
   <si>
@@ -224,12 +248,18 @@
     <t xml:space="preserve"> no trajo nada</t>
   </si>
   <si>
+    <t xml:space="preserve">probar liquidos, mejorar prototipo y ladron de joules, conectar led, le di toroide</t>
+  </si>
+  <si>
     <t xml:space="preserve">Paloma Marianella</t>
   </si>
   <si>
     <t xml:space="preserve">FARIAS RUIZ</t>
   </si>
   <si>
+    <t xml:space="preserve">subir un prototipo </t>
+  </si>
+  <si>
     <t xml:space="preserve">León</t>
   </si>
   <si>
@@ -255,6 +285,9 @@
   </si>
   <si>
     <t xml:space="preserve">no tenemos material</t>
+  </si>
+  <si>
+    <t xml:space="preserve">probar baldoza con ladron de joules</t>
   </si>
   <si>
     <t xml:space="preserve">Thiago Ezquiel</t>
@@ -383,7 +416,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -401,6 +434,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -707,17 +744,24 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="5" min="5" style="1" width="8.62"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="11" min="6" style="1" width="8.79"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="1" width="13.32"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="21" min="13" style="1" width="8.79"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="8.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="63.84"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="25" min="24" style="1" width="8.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="53.33"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="28" min="27" style="1" width="8.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="63.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="60.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="81.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="37" style="1" width="18.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16328" style="1" width="10.58"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="22" min="13" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="23" min="23" style="1" width="63.84"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="25" min="24" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="26" min="26" style="1" width="53.33"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="28" min="27" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="29" min="29" style="1" width="63.84"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="31" min="30" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="32" min="32" style="1" width="60.08"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="35" min="33" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="36" min="36" style="1" width="81.26"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="37" min="37" style="1" width="18.33"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="38" min="38" style="1" width="63.23"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="40" min="39" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="41" min="41" style="1" width="63.23"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="43" min="42" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="65.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16334" style="1" width="10.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -832,66 +876,82 @@
         <v>4</v>
       </c>
       <c r="AM1" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="AN1" s="2" t="n">
-        <v>46248</v>
-      </c>
-      <c r="AO1" s="2" t="n">
-        <v>46255</v>
+        <v>46262</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="AP1" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="AQ1" s="2" t="n">
         <v>46269</v>
       </c>
-      <c r="AR1" s="2" t="n">
+      <c r="AQ1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AS1" s="2" t="n">
         <v>46276</v>
       </c>
-      <c r="AS1" s="2" t="n">
+      <c r="AT1" s="2" t="n">
         <v>46283</v>
       </c>
-      <c r="AT1" s="2" t="n">
+      <c r="AU1" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="AU1" s="2" t="n">
+      <c r="AV1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AX1" s="2"/>
+      <c r="AY1" s="2" t="n">
         <v>46297</v>
       </c>
-      <c r="AV1" s="2" t="n">
+      <c r="AZ1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="BA1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="BB1" s="2" t="n">
         <v>46304</v>
       </c>
-      <c r="AW1" s="2" t="n">
+      <c r="BC1" s="2" t="n">
         <v>46311</v>
       </c>
-      <c r="AX1" s="2" t="n">
+      <c r="BD1" s="2" t="n">
         <v>46318</v>
       </c>
-      <c r="AY1" s="2" t="n">
+      <c r="BE1" s="2" t="n">
         <v>46325</v>
       </c>
-      <c r="AZ1" s="2" t="n">
+      <c r="BF1" s="2" t="n">
         <v>46332</v>
       </c>
-      <c r="BA1" s="2" t="n">
+      <c r="BG1" s="2" t="n">
         <v>46339</v>
       </c>
-      <c r="BB1" s="2" t="n">
+      <c r="BH1" s="2" t="n">
         <v>46346</v>
       </c>
-      <c r="BC1" s="2" t="n">
+      <c r="BI1" s="2" t="n">
         <v>46353</v>
       </c>
-      <c r="BD1" s="2" t="n">
+      <c r="BJ1" s="2" t="n">
         <v>46360</v>
       </c>
-      <c r="BE1" s="2" t="n">
+      <c r="BK1" s="2" t="n">
         <v>46367</v>
       </c>
-      <c r="BF1" s="2" t="n">
+      <c r="BL1" s="2" t="n">
         <v>46374</v>
       </c>
-      <c r="BG1" s="2" t="n">
+      <c r="BM1" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -900,42 +960,42 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q2" s="3" t="n">
         <f aca="false">COUNTIF(E2:P2,"P")</f>
@@ -958,99 +1018,138 @@
         <v>TEA</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y2" s="1" t="n">
         <v>9</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB2" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AC2" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE2" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AF2" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AG2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH2" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI2" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AJ2" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="AK2" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="BH2" s="2"/>
-      <c r="BI2" s="2"/>
-      <c r="BJ2" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="AM2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN2" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="AP2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AT2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ2" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="BN2" s="2"/>
+      <c r="BO2" s="2"/>
+      <c r="BP2" s="2"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q3" s="3" t="n">
         <f aca="false">COUNTIF(E3:P3,"P")</f>
@@ -1073,45 +1172,69 @@
         <v>TEA</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y3" s="3" t="n">
         <v>9</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB3" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE3" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH3" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI3" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AK3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="XCZ3" s="1"/>
-      <c r="XDA3" s="1"/>
-      <c r="XDB3" s="1"/>
-      <c r="XDC3" s="1"/>
-      <c r="XDD3" s="1"/>
-      <c r="XDE3" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="AM3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ3" s="1"/>
+      <c r="AR3" s="1"/>
+      <c r="AT3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX3" s="1"/>
+      <c r="AY3" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ3" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA3" s="0" t="n">
+        <v>6</v>
+      </c>
       <c r="XDF3" s="1"/>
       <c r="XDG3" s="1"/>
       <c r="XDH3" s="1"/>
@@ -1169,40 +1292,40 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q4" s="3" t="n">
         <f aca="false">COUNTIF(E4:P4,"P")</f>
@@ -1225,45 +1348,69 @@
         <v>TEA</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y4" s="3" t="n">
         <v>9</v>
       </c>
       <c r="AA4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB4" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AD4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE4" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH4" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI4" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ4" s="1"/>
-      <c r="XDA4" s="1"/>
-      <c r="XDB4" s="1"/>
-      <c r="XDC4" s="1"/>
-      <c r="XDD4" s="1"/>
-      <c r="XDE4" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
+      <c r="AT4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV4" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW4" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX4" s="1"/>
+      <c r="AY4" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ4" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA4" s="0" t="n">
+        <v>6</v>
+      </c>
       <c r="XDF4" s="1"/>
       <c r="XDG4" s="1"/>
       <c r="XDH4" s="1"/>
@@ -1316,45 +1463,45 @@
       <c r="XFC4" s="1"/>
       <c r="XFD4" s="1"/>
     </row>
-    <row r="5" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="1" customFormat="true" ht="18.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q5" s="3" t="n">
         <f aca="false">COUNTIF(E5:P5,"P")</f>
@@ -1377,95 +1524,122 @@
         <v>TEA</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y5" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB5" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AD5" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE5" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI5" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV5" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW5" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY5" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ5" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA5" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="P6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q6" s="5" t="n">
+      <c r="F6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="6" t="n">
         <f aca="false">COUNTIF(E6:P6,"P")</f>
         <v>7</v>
       </c>
-      <c r="R6" s="6" t="n">
+      <c r="R6" s="7" t="n">
         <f aca="false">COUNTIF(E6:P6,"A")</f>
         <v>2</v>
       </c>
-      <c r="S6" s="5" t="n">
+      <c r="S6" s="6" t="n">
         <f aca="false">SUM(Q6:R6)</f>
         <v>9</v>
       </c>
@@ -1477,38 +1651,66 @@
         <f aca="false">IF(T6&gt;6,"TEA",IF(T6&gt;3,"TEP","TED"))</f>
         <v>TEA</v>
       </c>
-      <c r="V6" s="6" t="s">
-        <v>13</v>
+      <c r="V6" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y6" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB6" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AD6" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE6" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AG6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="AH6" s="6" t="s">
-        <v>13</v>
+      <c r="AG6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH6" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="AI6" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN6" s="7"/>
+      <c r="AP6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV6" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW6" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY6" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ6" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA6" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1516,40 +1718,40 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q7" s="3" t="n">
         <f aca="false">COUNTIF(E7:P7,"P")</f>
@@ -1572,81 +1774,108 @@
         <v>TEA</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y7" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AA7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB7" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AD7" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE7" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AG7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI7" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AU7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY7" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ7" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA7" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
-    <row r="8" s="3" customFormat="true" ht="33.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" s="3" customFormat="true" ht="15.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q8" s="3" t="n">
         <f aca="false">COUNTIF(E8:P8,"P")</f>
@@ -1669,60 +1898,90 @@
         <v>TEA</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y8" s="3" t="n">
         <v>3</v>
       </c>
       <c r="Z8" s="3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="AA8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE8" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AF8" s="3" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="AG8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI8" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="AJ8" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="AL8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM8" s="7"/>
-      <c r="XCZ8" s="1"/>
-      <c r="XDA8" s="1"/>
-      <c r="XDB8" s="1"/>
-      <c r="XDC8" s="1"/>
-      <c r="XDD8" s="1"/>
-      <c r="XDE8" s="1"/>
+      <c r="AJ8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK8" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN8" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AP8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AT8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX8" s="1"/>
+      <c r="AY8" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ8" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA8" s="0" t="n">
+        <v>8</v>
+      </c>
       <c r="XDF8" s="1"/>
       <c r="XDG8" s="1"/>
       <c r="XDH8" s="1"/>
@@ -1780,42 +2039,42 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q9" s="3" t="n">
         <f aca="false">COUNTIF(E9:P9,"P")</f>
@@ -1838,49 +2097,75 @@
         <v>TEA</v>
       </c>
       <c r="V9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="Z9" s="1"/>
       <c r="AA9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB9" s="3" t="n">
         <v>7</v>
       </c>
       <c r="AC9" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="AD9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE9" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AF9" s="1"/>
       <c r="AG9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH9" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI9" s="3" t="n">
         <v>10</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ9" s="1"/>
-      <c r="XDA9" s="1"/>
-      <c r="XDB9" s="1"/>
-      <c r="XDC9" s="1"/>
-      <c r="XDD9" s="1"/>
-      <c r="XDE9" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ9" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR9" s="1"/>
+      <c r="AT9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX9" s="1"/>
+      <c r="AY9" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA9" s="0" t="n">
+        <v>8</v>
+      </c>
       <c r="XDF9" s="1"/>
       <c r="XDG9" s="1"/>
       <c r="XDH9" s="1"/>
@@ -1938,41 +2223,41 @@
         <v>18</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q10" s="3" t="n">
         <f aca="false">COUNTIF(E10:P10,"P")</f>
@@ -1995,45 +2280,72 @@
         <v>TEA</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y10" s="3" t="n">
         <v>3</v>
       </c>
       <c r="AA10" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB10" s="3" t="n">
         <v>7</v>
       </c>
       <c r="AD10" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE10" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI10" s="3" t="n">
         <v>10</v>
       </c>
       <c r="AK10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ10" s="1"/>
-      <c r="XDA10" s="1"/>
-      <c r="XDB10" s="1"/>
-      <c r="XDC10" s="1"/>
-      <c r="XDD10" s="1"/>
-      <c r="XDE10" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN10" s="1"/>
+      <c r="AP10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ10" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR10" s="1"/>
+      <c r="AT10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV10" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW10" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX10" s="1"/>
+      <c r="AY10" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ10" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA10" s="0" t="n">
+        <v>8</v>
+      </c>
       <c r="XDF10" s="1"/>
       <c r="XDG10" s="1"/>
       <c r="XDH10" s="1"/>
@@ -2091,40 +2403,40 @@
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q11" s="3" t="n">
         <f aca="false">COUNTIF(E11:P11,"P")</f>
@@ -2147,52 +2459,88 @@
         <v>TEA</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y11" s="1" t="n">
         <v>5</v>
       </c>
       <c r="Z11" s="3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB11" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AD11" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE11" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AF11" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="AG11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH11" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AJ11" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="AK11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AL11" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
+      </c>
+      <c r="AM11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AP11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AR11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AT11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW11" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY11" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ11" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA11" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2200,41 +2548,41 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L12" s="3"/>
       <c r="M12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q12" s="3" t="n">
         <f aca="false">COUNTIF(E12:P12,"P")</f>
@@ -2257,43 +2605,74 @@
         <v>TEA</v>
       </c>
       <c r="V12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y12" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AB12" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AD12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE12" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AF12" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="AG12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH12" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI12" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AJ12" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN12" s="3"/>
+      <c r="AP12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ12" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AT12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW12" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY12" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ12" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA12" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2301,42 +2680,42 @@
         <v>17</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q13" s="3" t="n">
         <f aca="false">COUNTIF(E13:P13,"P")</f>
@@ -2359,37 +2738,67 @@
         <v>TEA</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="X13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y13" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AA13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AD13" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE13" s="1" t="n">
         <v>9</v>
       </c>
       <c r="AG13" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH13" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AI13" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AK13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ13" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AT13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV13" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW13" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY13" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="AZ13" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA13" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="14" s="3" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2397,41 +2806,41 @@
         <v>6</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q14" s="3" t="n">
         <f aca="false">COUNTIF(E14:P14,"P")</f>
@@ -2454,156 +2863,185 @@
         <v>TEA</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W14" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="X14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y14" s="3" t="n">
         <v>7</v>
       </c>
       <c r="Z14" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="AA14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AB14" s="3" t="n">
         <v>5</v>
       </c>
       <c r="AC14" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="AD14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE14" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AF14" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="AG14" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="AJ14" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AK14" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="AK14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AL14" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="XCZ14" s="1"/>
-      <c r="XDA14" s="1"/>
-      <c r="XDB14" s="5"/>
-      <c r="XDC14" s="5"/>
-      <c r="XDD14" s="5"/>
-      <c r="XDE14" s="5"/>
-      <c r="XDF14" s="5"/>
-      <c r="XDG14" s="5"/>
-      <c r="XDH14" s="5"/>
-      <c r="XDI14" s="5"/>
-      <c r="XDJ14" s="5"/>
-      <c r="XDK14" s="5"/>
-      <c r="XDL14" s="5"/>
-      <c r="XDM14" s="5"/>
-      <c r="XDN14" s="5"/>
-      <c r="XDO14" s="5"/>
-      <c r="XDP14" s="5"/>
-      <c r="XDQ14" s="5"/>
-      <c r="XDR14" s="5"/>
-      <c r="XDS14" s="5"/>
-      <c r="XDT14" s="5"/>
-      <c r="XDU14" s="5"/>
-      <c r="XDV14" s="5"/>
-      <c r="XDW14" s="5"/>
-      <c r="XDX14" s="5"/>
-      <c r="XDY14" s="5"/>
-      <c r="XDZ14" s="5"/>
-      <c r="XEA14" s="5"/>
-      <c r="XEB14" s="5"/>
-      <c r="XEC14" s="5"/>
-      <c r="XED14" s="5"/>
-      <c r="XEE14" s="5"/>
-      <c r="XEF14" s="5"/>
-      <c r="XEG14" s="5"/>
-      <c r="XEH14" s="5"/>
-      <c r="XEI14" s="5"/>
-      <c r="XEJ14" s="5"/>
-      <c r="XEK14" s="5"/>
-      <c r="XEL14" s="5"/>
-      <c r="XEM14" s="5"/>
-      <c r="XEN14" s="5"/>
-      <c r="XEO14" s="5"/>
-      <c r="XEP14" s="5"/>
-      <c r="XEQ14" s="5"/>
-      <c r="XER14" s="5"/>
-      <c r="XES14" s="5"/>
-      <c r="XET14" s="5"/>
-      <c r="XEU14" s="5"/>
-      <c r="XEV14" s="5"/>
-      <c r="XEW14" s="5"/>
-      <c r="XEX14" s="5"/>
-      <c r="XEY14" s="5"/>
-      <c r="XEZ14" s="5"/>
-      <c r="XFA14" s="5"/>
-      <c r="XFB14" s="5"/>
-      <c r="XFC14" s="5"/>
-      <c r="XFD14" s="5"/>
+      <c r="AL14" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN14" s="1"/>
+      <c r="AP14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ14" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR14" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="AT14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW14" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX14" s="1"/>
+      <c r="AY14" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA14" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="XDF14" s="1"/>
+      <c r="XDG14" s="1"/>
+      <c r="XDH14" s="1"/>
+      <c r="XDI14" s="1"/>
+      <c r="XDJ14" s="1"/>
+      <c r="XDK14" s="6"/>
+      <c r="XDL14" s="6"/>
+      <c r="XDM14" s="6"/>
+      <c r="XDN14" s="6"/>
+      <c r="XDO14" s="6"/>
+      <c r="XDP14" s="6"/>
+      <c r="XDQ14" s="6"/>
+      <c r="XDR14" s="6"/>
+      <c r="XDS14" s="6"/>
+      <c r="XDT14" s="6"/>
+      <c r="XDU14" s="6"/>
+      <c r="XDV14" s="6"/>
+      <c r="XDW14" s="6"/>
+      <c r="XDX14" s="6"/>
+      <c r="XDY14" s="6"/>
+      <c r="XDZ14" s="6"/>
+      <c r="XEA14" s="6"/>
+      <c r="XEB14" s="6"/>
+      <c r="XEC14" s="6"/>
+      <c r="XED14" s="6"/>
+      <c r="XEE14" s="6"/>
+      <c r="XEF14" s="6"/>
+      <c r="XEG14" s="6"/>
+      <c r="XEH14" s="6"/>
+      <c r="XEI14" s="6"/>
+      <c r="XEJ14" s="6"/>
+      <c r="XEK14" s="6"/>
+      <c r="XEL14" s="6"/>
+      <c r="XEM14" s="6"/>
+      <c r="XEN14" s="6"/>
+      <c r="XEO14" s="6"/>
+      <c r="XEP14" s="6"/>
+      <c r="XEQ14" s="6"/>
+      <c r="XER14" s="6"/>
+      <c r="XES14" s="6"/>
+      <c r="XET14" s="6"/>
+      <c r="XEU14" s="6"/>
+      <c r="XEV14" s="6"/>
+      <c r="XEW14" s="6"/>
+      <c r="XEX14" s="6"/>
+      <c r="XEY14" s="6"/>
+      <c r="XEZ14" s="6"/>
+      <c r="XFA14" s="6"/>
+      <c r="XFB14" s="6"/>
+      <c r="XFC14" s="6"/>
+      <c r="XFD14" s="6"/>
     </row>
-    <row r="15" s="6" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="7" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J15" s="1"/>
       <c r="K15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="3" t="n">
         <f aca="false">COUNTIF(E15:P15,"P")</f>
@@ -2626,45 +3064,75 @@
         <v>TEA</v>
       </c>
       <c r="V15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="X15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y15" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="AA15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="AB15" s="6" t="n">
+      <c r="AA15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB15" s="7" t="n">
         <v>5</v>
       </c>
       <c r="AD15" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE15" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AF15" s="1"/>
       <c r="AG15" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="AI15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="AI15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AK15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ15" s="1"/>
-      <c r="XDA15" s="1"/>
-      <c r="XDB15" s="1"/>
-      <c r="XDC15" s="1"/>
-      <c r="XDD15" s="1"/>
-      <c r="XDE15" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN15" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AO15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AQ15" s="1"/>
+      <c r="AR15" s="1"/>
+      <c r="AT15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW15" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX15" s="1"/>
+      <c r="AY15" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA15" s="0" t="n">
+        <v>5</v>
+      </c>
       <c r="XDF15" s="1"/>
       <c r="XDG15" s="1"/>
       <c r="XDH15" s="1"/>
@@ -2722,40 +3190,40 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="E16" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q16" s="3" t="n">
         <f aca="false">COUNTIF(E16:P16,"P")</f>
@@ -2778,46 +3246,70 @@
         <v>TEA</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W16" s="1"/>
       <c r="X16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Y16" s="3" t="n">
         <v>7</v>
       </c>
       <c r="AA16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB16" s="3" t="n">
         <v>5</v>
       </c>
       <c r="AD16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE16" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH16" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="AK16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ16" s="1"/>
-      <c r="XDA16" s="1"/>
-      <c r="XDB16" s="1"/>
-      <c r="XDC16" s="1"/>
-      <c r="XDD16" s="1"/>
-      <c r="XDE16" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ16" s="1"/>
+      <c r="AR16" s="1"/>
+      <c r="AT16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV16" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW16" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX16" s="1"/>
+      <c r="AY16" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA16" s="0" t="n">
+        <v>5</v>
+      </c>
       <c r="XDF16" s="1"/>
       <c r="XDG16" s="1"/>
       <c r="XDH16" s="1"/>
@@ -2875,41 +3367,41 @@
         <v>12</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L17" s="1"/>
       <c r="M17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q17" s="3" t="n">
         <f aca="false">COUNTIF(E17:P17,"P")</f>
@@ -2932,45 +3424,70 @@
         <v>TEA</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y17" s="3" t="n">
         <v>7</v>
       </c>
       <c r="AA17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB17" s="3" t="n">
         <v>5</v>
       </c>
       <c r="AD17" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE17" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH17" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="AK17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="XCZ17" s="1"/>
-      <c r="XDA17" s="1"/>
-      <c r="XDB17" s="1"/>
-      <c r="XDC17" s="1"/>
-      <c r="XDD17" s="1"/>
-      <c r="XDE17" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="AM17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN17" s="1"/>
+      <c r="AP17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ17" s="1"/>
+      <c r="AR17" s="1"/>
+      <c r="AT17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AV17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW17" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX17" s="1"/>
+      <c r="AY17" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA17" s="0" t="n">
+        <v>5</v>
+      </c>
       <c r="XDF17" s="1"/>
       <c r="XDG17" s="1"/>
       <c r="XDH17" s="1"/>
@@ -3028,41 +3545,41 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L18" s="3"/>
       <c r="M18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q18" s="3" t="n">
         <f aca="false">COUNTIF(E18:P18,"P")</f>
@@ -3085,55 +3602,94 @@
         <v>TEA</v>
       </c>
       <c r="V18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W18" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="X18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="Z18" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AA18" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB18" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AC18" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AD18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE18" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AF18" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AG18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH18" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AJ18" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AK18" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AL18" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
+      </c>
+      <c r="AM18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN18" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AO18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="AP18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ18" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR18" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AT18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV18" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW18" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AY18" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ18" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="BA18" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3141,43 +3697,43 @@
         <v>10</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L19" s="3"/>
       <c r="M19" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q19" s="3" t="n">
         <f aca="false">COUNTIF(E19:P19,"P")</f>
@@ -3200,37 +3756,64 @@
         <v>TEA</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AA19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB19" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AD19" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE19" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AK19" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AU19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV19" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW19" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AY19" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ19" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="BA19" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3238,40 +3821,40 @@
         <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="Q20" s="3" t="n">
         <f aca="false">COUNTIF(E20:P20,"P")</f>
@@ -3294,37 +3877,65 @@
         <v>TEA</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AA20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB20" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AD20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE20" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AG20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AH20" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AI20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AK20" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN20" s="3"/>
+      <c r="AP20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT20" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AU20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV20" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW20" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AY20" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ20" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="BA20" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3332,40 +3943,40 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q21" s="3" t="n">
         <f aca="false">COUNTIF(E21:P21,"P")</f>
@@ -3388,43 +3999,83 @@
         <v>TEA</v>
       </c>
       <c r="V21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="X21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y21" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AA21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB21" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AD21" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE21" s="1" t="n">
         <v>7</v>
       </c>
       <c r="AG21" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AH21" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AI21" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AK21" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="AM21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV21" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW21" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AY21" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ21" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="BA21" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AT22" s="1" t="n">
+        <f aca="false">COUNTIF(AT2:AT21,"P")</f>
+        <v>17</v>
+      </c>
+      <c r="AU22" s="1" t="n">
+        <f aca="false">COUNTIF(AU2:AU21,"P")</f>
+        <v>19</v>
+      </c>
+      <c r="AY22" s="1" t="n">
+        <f aca="false">COUNTIF(AY2:AY21,"P")</f>
+        <v>19</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>5</v>
@@ -3481,23 +4132,25 @@
         <f aca="false">COUNTIF(AD2:AD22,"P")</f>
         <v>20</v>
       </c>
-      <c r="AE23" s="1"/>
       <c r="AG23" s="1" t="n">
         <f aca="false">COUNTIF(AG2:AG22,"P")</f>
         <v>14</v>
       </c>
-      <c r="AH23" s="1"/>
       <c r="AK23" s="1" t="n">
         <f aca="false">COUNTIF(AK2:AK22,"P")</f>
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="AP23" s="1" t="n">
+        <f aca="false">COUNTIF(AP2:AP22,"P")</f>
+        <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C24" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E24" s="1" t="n">
         <f aca="false">COUNTIF(E3:E17,"M")</f>
@@ -3551,23 +4204,25 @@
         <f aca="false">COUNTIF(AD3:AD17,"M")</f>
         <v>0</v>
       </c>
-      <c r="AE24" s="1"/>
       <c r="AG24" s="1" t="n">
         <f aca="false">COUNTIF(AG3:AG17,"M")</f>
         <v>0</v>
       </c>
-      <c r="AH24" s="1"/>
       <c r="AK24" s="1" t="n">
         <f aca="false">COUNTIF(AK3:AK17,"M")</f>
         <v>0</v>
       </c>
+      <c r="AP24" s="1" t="n">
+        <f aca="false">COUNTIF(AP3:AP17,"M")</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="1" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="E25" s="1" t="n">
         <f aca="false">COUNTIF(E3:E17,"T")</f>
@@ -3621,14 +4276,16 @@
         <f aca="false">COUNTIF(AD3:AD17,"T")</f>
         <v>0</v>
       </c>
-      <c r="AE25" s="1"/>
       <c r="AG25" s="1" t="n">
         <f aca="false">COUNTIF(AG3:AG17,"T")</f>
         <v>0</v>
       </c>
-      <c r="AH25" s="1"/>
       <c r="AK25" s="1" t="n">
         <f aca="false">COUNTIF(AK3:AK17,"T")</f>
+        <v>0</v>
+      </c>
+      <c r="AP25" s="1" t="n">
+        <f aca="false">COUNTIF(AP3:AP17,"T")</f>
         <v>0</v>
       </c>
     </row>
@@ -3688,15 +4345,17 @@
         <f aca="false">SUM(AD23:AD25)</f>
         <v>20</v>
       </c>
-      <c r="AE26" s="1"/>
       <c r="AG26" s="1" t="n">
         <f aca="false">SUM(AG23:AG25)</f>
         <v>14</v>
       </c>
-      <c r="AH26" s="1"/>
       <c r="AK26" s="1" t="n">
         <f aca="false">SUM(AK23:AK25)</f>
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="AP26" s="1" t="n">
+        <f aca="false">SUM(AP23:AP25)</f>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -3779,22 +4438,22 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3802,13 +4461,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>10</v>
@@ -3835,13 +4494,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>7</v>
@@ -3868,13 +4527,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>1</v>
@@ -3901,13 +4560,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>1</v>
@@ -3934,13 +4593,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>9</v>
@@ -3967,13 +4626,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>10</v>
@@ -4000,13 +4659,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>1</v>
@@ -4033,13 +4692,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>8</v>
@@ -4066,13 +4725,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>10</v>
@@ -4099,13 +4758,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>9</v>
@@ -4129,13 +4788,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>9</v>
@@ -4159,13 +4818,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>9</v>
@@ -4189,13 +4848,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>8</v>
@@ -4219,13 +4878,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>8</v>
@@ -4249,13 +4908,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>8</v>
@@ -4279,13 +4938,13 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>8</v>
@@ -4309,13 +4968,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>9</v>
@@ -4339,13 +4998,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>9</v>
@@ -4369,13 +5028,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>9</v>
@@ -4399,13 +5058,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>9</v>

</xml_diff>